<commit_message>
Add Bernard river station
</commit_message>
<xml_diff>
--- a/Resources/Metadata.xlsx
+++ b/Resources/Metadata.xlsx
@@ -1,35 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ulavaldti-my.sharepoint.com/personal/anthi182_ulaval_ca/Documents/Documents/GitHub/Ro2_data_worflow/Resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:1_{6983D7D3-A322-4149-A22B-9F8F3383839B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63146463-5547-4E8E-BC2B-246FB77354AB}"/>
+  <xr:revisionPtr revIDLastSave="87" documentId="13_ncr:1_{6983D7D3-A322-4149-A22B-9F8F3383839B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CC1C3CED-85C4-449C-97A3-F72140D718BF}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="3" xr2:uid="{70FED0F5-DA18-6E4C-8F4F-A74F12345264}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{70FED0F5-DA18-6E4C-8F4F-A74F12345264}"/>
   </bookViews>
   <sheets>
-    <sheet name="Berge" sheetId="3" r:id="rId1"/>
-    <sheet name="Reservoir" sheetId="4" r:id="rId2"/>
-    <sheet name="Romaine-2 thermistors" sheetId="6" r:id="rId3"/>
-    <sheet name="Bernard_lake" sheetId="8" r:id="rId4"/>
-    <sheet name="Bernard lake thermistors" sheetId="9" r:id="rId5"/>
-    <sheet name="Foret" sheetId="5" r:id="rId6"/>
-    <sheet name="Foret_neige" sheetId="11" r:id="rId7"/>
-    <sheet name="Natashquan" sheetId="7" r:id="rId8"/>
-    <sheet name="Juvenile" sheetId="12" r:id="rId9"/>
-    <sheet name="Sapling" sheetId="13" r:id="rId10"/>
-    <sheet name="Regeneration" sheetId="14" r:id="rId11"/>
-    <sheet name="Neige" sheetId="15" r:id="rId12"/>
-    <sheet name="Juvenile_Schematics_2015_2020" sheetId="17" r:id="rId13"/>
-    <sheet name="Juvenile_Schematics_2021" sheetId="16" r:id="rId14"/>
-    <sheet name="Sapling_Schematics_2015_2022" sheetId="18" r:id="rId15"/>
-    <sheet name="Sapling Schematics_2023" sheetId="19" r:id="rId16"/>
-    <sheet name="Regeneration_Schematics_2024" sheetId="20" r:id="rId17"/>
+    <sheet name="Bernard Lake" sheetId="8" r:id="rId1"/>
+    <sheet name="Bernard Lake thermistors" sheetId="9" r:id="rId2"/>
+    <sheet name="Bernard River" sheetId="21" r:id="rId3"/>
+    <sheet name="Bernard Spruce Moss" sheetId="5" r:id="rId4"/>
+    <sheet name="Bernard Spruce Moss Snow" sheetId="11" r:id="rId5"/>
+    <sheet name="Romaine-2 Reservoir Raft" sheetId="4" r:id="rId6"/>
+    <sheet name="Romaine-2 Reservoir Shore" sheetId="3" r:id="rId7"/>
+    <sheet name="Romaine-2 Reservoir Thermistors" sheetId="6" r:id="rId8"/>
+    <sheet name="Natashquan" sheetId="7" r:id="rId9"/>
+    <sheet name="Juvenile" sheetId="12" r:id="rId10"/>
+    <sheet name="Sapling" sheetId="13" r:id="rId11"/>
+    <sheet name="Regeneration" sheetId="14" r:id="rId12"/>
+    <sheet name="Neige" sheetId="15" r:id="rId13"/>
+    <sheet name="Juvenile_Schematics_2015_2020" sheetId="17" r:id="rId14"/>
+    <sheet name="Juvenile_Schematics_2021" sheetId="16" r:id="rId15"/>
+    <sheet name="Sapling_Schematics_2015_2022" sheetId="18" r:id="rId16"/>
+    <sheet name="Sapling Schematics_2023" sheetId="19" r:id="rId17"/>
+    <sheet name="Regeneration_Schematics_2024" sheetId="20" r:id="rId18"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="749" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="765" uniqueCount="254">
   <si>
     <t>Instrument</t>
   </si>
@@ -790,6 +791,33 @@
   </si>
   <si>
     <t>Pressure transducer</t>
+  </si>
+  <si>
+    <t>Bernard river</t>
+  </si>
+  <si>
+    <t>SonTek IQ+</t>
+  </si>
+  <si>
+    <t>Sommer RQ30+</t>
+  </si>
+  <si>
+    <t>Doppler</t>
+  </si>
+  <si>
+    <t>Radar</t>
+  </si>
+  <si>
+    <t>Hobo U20L</t>
+  </si>
+  <si>
+    <t>0m reference is arbitrary level. Always under water</t>
+  </si>
+  <si>
+    <t>0 and 0.9</t>
+  </si>
+  <si>
+    <t>One sensor at the bottom of the scale (0m), and one at the tower foot (~0.9m)</t>
   </si>
 </sst>
 </file>
@@ -1636,7 +1664,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="150">
+  <cellXfs count="154">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1842,6 +1870,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="56" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="45" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="57" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1908,9 +1939,18 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="56" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="45" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="57" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1930,6 +1970,61 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>292100</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1362074</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>25863</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5D4297F3-F50C-4418-B164-908F7C0B23B7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="292100" y="1568450"/>
+          <a:ext cx="4879974" cy="3200863"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -2083,7 +2178,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -2237,7 +2332,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -2452,7 +2547,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -2606,7 +2701,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -3121,39 +3216,33 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE44D4E6-1DC8-5846-9613-DEB0E908B686}">
-  <dimension ref="B1:J16"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B1D1867-B0BA-4CF9-B964-CDDBB5D9DD8C}">
+  <dimension ref="B1:H18"/>
   <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="17.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25.75" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.75" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="7" max="7" width="11.25" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.33203125" customWidth="1"/>
-    <col min="9" max="9" width="25.33203125" customWidth="1"/>
-    <col min="10" max="10" width="20.5" customWidth="1"/>
+    <col min="4" max="4" width="24.08203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.58203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-    </row>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B2" s="125" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="126"/>
-      <c r="D2" s="126"/>
-      <c r="E2" s="127"/>
-      <c r="G2" s="7" t="s">
+    <row r="1" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="2" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B2" s="128" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="129"/>
+      <c r="D2" s="129"/>
+      <c r="E2" s="130"/>
+      <c r="G2" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="H2" s="8">
-        <v>50.653801000000001</v>
-      </c>
-    </row>
-    <row r="3" spans="2:10" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="H2" s="15">
+        <v>50.861454700000003</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B3" s="21" t="s">
         <v>0</v>
       </c>
@@ -3161,19 +3250,19 @@
         <v>107</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E3" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="G3" s="13" t="s">
+      <c r="G3" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="3">
-        <v>-63.259498600000001</v>
-      </c>
-    </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="H3" s="2">
+        <v>-63.389840900000003</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B4" s="23" t="s">
         <v>1</v>
       </c>
@@ -3181,35 +3270,35 @@
         <v>108</v>
       </c>
       <c r="D4" s="19">
-        <v>8</v>
+        <v>0.8</v>
       </c>
       <c r="E4" s="11"/>
     </row>
-    <row r="5" spans="2:10" ht="31" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:8" ht="31" x14ac:dyDescent="0.35">
       <c r="B5" s="24" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="64" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="D5" s="20">
-        <v>7.25</v>
+        <v>4.3</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.35">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B6" s="23" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="19"/>
       <c r="D6" s="19">
-        <v>7.25</v>
+        <v>4.3</v>
       </c>
       <c r="E6" s="11"/>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B7" s="24" t="s">
         <v>5</v>
       </c>
@@ -3217,125 +3306,521 @@
         <v>110</v>
       </c>
       <c r="D7" s="20">
-        <v>7.25</v>
+        <v>4.3</v>
       </c>
       <c r="E7" s="1"/>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B8" s="23" t="s">
-        <v>92</v>
+        <v>7</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>242</v>
+        <v>111</v>
       </c>
       <c r="D8" s="19">
-        <v>2.5</v>
-      </c>
-      <c r="E8" s="60" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.35">
+        <v>3.9</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B9" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>112</v>
+      </c>
+      <c r="D9" s="20">
+        <v>0.8</v>
+      </c>
+      <c r="E9" s="27"/>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B10" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="D10" s="19">
+        <v>2</v>
+      </c>
+      <c r="E10" s="11"/>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B11" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>114</v>
+      </c>
+      <c r="D11" s="20">
+        <v>1.2</v>
+      </c>
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B12" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="D12" s="19">
+        <v>1</v>
+      </c>
+      <c r="E12" s="11"/>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B13" s="125" t="s">
+        <v>243</v>
+      </c>
+      <c r="C13" s="126" t="s">
+        <v>244</v>
+      </c>
+      <c r="D13" s="126">
+        <v>1.2</v>
+      </c>
+      <c r="E13" s="127"/>
+    </row>
+    <row r="14" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B14" s="25" t="s">
+        <v>83</v>
+      </c>
+      <c r="C14" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="D14" s="26">
+        <v>1</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B16" s="131" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" s="132"/>
+      <c r="D16" s="132"/>
+      <c r="E16" s="133"/>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B17" s="21"/>
+      <c r="C17" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="E17" s="22" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B18" s="25" t="s">
+        <v>5</v>
+      </c>
+      <c r="C18" s="26">
+        <v>-37.5</v>
+      </c>
+      <c r="D18" s="26">
+        <v>5.5</v>
+      </c>
+      <c r="E18" s="12">
         <v>7</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>111</v>
-      </c>
-      <c r="D9" s="20">
-        <v>6.3</v>
-      </c>
-      <c r="E9" s="1"/>
-    </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B10" s="23" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" s="19" t="s">
-        <v>112</v>
-      </c>
-      <c r="D10" s="19">
-        <v>5.2</v>
-      </c>
-      <c r="E10" s="61" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B11" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="20" t="s">
-        <v>113</v>
-      </c>
-      <c r="D11" s="20">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="E11" s="1"/>
-    </row>
-    <row r="12" spans="2:10" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="C12" s="26" t="s">
-        <v>115</v>
-      </c>
-      <c r="D12" s="26">
-        <v>0.9</v>
-      </c>
-      <c r="E12" s="12"/>
-    </row>
-    <row r="13" spans="2:10" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="G13" s="28"/>
-      <c r="H13" s="28"/>
-      <c r="I13" s="28"/>
-      <c r="J13" s="28"/>
-    </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B14" s="128" t="s">
-        <v>33</v>
-      </c>
-      <c r="C14" s="129"/>
-      <c r="D14" s="129"/>
-      <c r="E14" s="130"/>
-    </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B15" s="21"/>
-      <c r="C15" s="18" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="E15" s="22" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="16" spans="2:10" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B16" s="25" t="s">
-        <v>5</v>
-      </c>
-      <c r="C16" s="26">
-        <v>26</v>
-      </c>
-      <c r="D16" s="26">
-        <v>-13.6</v>
-      </c>
-      <c r="E16" s="12">
-        <v>3</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="B16:E16"/>
   </mergeCells>
-  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87885471-7CC2-479B-9C76-A0AAB2D0375D}">
+  <dimension ref="B1:H28"/>
+  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="23.25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.75" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="40.25" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.25" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.83203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="2" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B2" s="128" t="s">
+        <v>131</v>
+      </c>
+      <c r="C2" s="129"/>
+      <c r="D2" s="129"/>
+      <c r="E2" s="130"/>
+      <c r="G2" s="115" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="116">
+        <v>47.287930000000003</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B3" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>122</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="G3" s="101" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="117">
+        <v>-71.167720000000003</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B4" s="112" t="s">
+        <v>198</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>200</v>
+      </c>
+      <c r="D4" s="119" t="s">
+        <v>175</v>
+      </c>
+      <c r="E4" s="114" t="s">
+        <v>172</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="H4" s="113" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B5" s="32" t="s">
+        <v>199</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>201</v>
+      </c>
+      <c r="D5" s="120" t="s">
+        <v>175</v>
+      </c>
+      <c r="E5" s="114" t="s">
+        <v>172</v>
+      </c>
+      <c r="G5" s="103" t="s">
+        <v>162</v>
+      </c>
+      <c r="H5" s="111" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B6" s="32" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="D6" s="120" t="s">
+        <v>171</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B7" s="32" t="s">
+        <v>209</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>206</v>
+      </c>
+      <c r="D7" s="120">
+        <v>1</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B8" s="32" t="s">
+        <v>207</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>206</v>
+      </c>
+      <c r="D8" s="120">
+        <v>2</v>
+      </c>
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B9" s="32" t="s">
+        <v>208</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>206</v>
+      </c>
+      <c r="D9" s="120">
+        <v>1</v>
+      </c>
+      <c r="E9" s="14"/>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B10" s="32" t="s">
+        <v>180</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>126</v>
+      </c>
+      <c r="D10" s="121" t="s">
+        <v>182</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B11" s="32" t="s">
+        <v>181</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>126</v>
+      </c>
+      <c r="D11" s="121" t="s">
+        <v>184</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B12" s="32" t="s">
+        <v>197</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>113</v>
+      </c>
+      <c r="D12" s="120" t="s">
+        <v>202</v>
+      </c>
+      <c r="E12" s="118" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B13" s="32" t="s">
+        <v>196</v>
+      </c>
+      <c r="C13" s="20" t="s">
+        <v>113</v>
+      </c>
+      <c r="D13" s="120" t="s">
+        <v>203</v>
+      </c>
+      <c r="E13" s="114" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B14" s="32" t="s">
+        <v>194</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>113</v>
+      </c>
+      <c r="D14" s="120" t="s">
+        <v>204</v>
+      </c>
+      <c r="E14" s="114" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B15" s="32" t="s">
+        <v>195</v>
+      </c>
+      <c r="C15" s="20" t="s">
+        <v>113</v>
+      </c>
+      <c r="D15" s="120" t="s">
+        <v>205</v>
+      </c>
+      <c r="E15" s="114" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B16" s="32" t="s">
+        <v>185</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="D16" s="120">
+        <v>-0.08</v>
+      </c>
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" spans="2:5" ht="31" x14ac:dyDescent="0.35">
+      <c r="B17" s="32" t="s">
+        <v>173</v>
+      </c>
+      <c r="C17" s="64" t="s">
+        <v>109</v>
+      </c>
+      <c r="D17" s="120" t="s">
+        <v>175</v>
+      </c>
+      <c r="E17" s="114" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" ht="31" x14ac:dyDescent="0.35">
+      <c r="B18" s="32" t="s">
+        <v>174</v>
+      </c>
+      <c r="C18" s="64" t="s">
+        <v>125</v>
+      </c>
+      <c r="D18" s="120" t="s">
+        <v>175</v>
+      </c>
+      <c r="E18" s="114" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B19" s="32" t="s">
+        <v>176</v>
+      </c>
+      <c r="C19" s="20" t="s">
+        <v>114</v>
+      </c>
+      <c r="D19" s="120" t="s">
+        <v>175</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B20" s="32" t="s">
+        <v>177</v>
+      </c>
+      <c r="C20" s="20" t="s">
+        <v>114</v>
+      </c>
+      <c r="D20" s="120" t="s">
+        <v>175</v>
+      </c>
+      <c r="E20" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B21" s="32" t="s">
+        <v>192</v>
+      </c>
+      <c r="C21" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="D21" s="120">
+        <v>8.5</v>
+      </c>
+      <c r="E21" s="14"/>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B22" s="32" t="s">
+        <v>193</v>
+      </c>
+      <c r="C22" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="D22" s="120">
+        <v>14.6</v>
+      </c>
+      <c r="E22" s="14"/>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B23" s="32" t="s">
+        <v>187</v>
+      </c>
+      <c r="C23" s="20" t="s">
+        <v>127</v>
+      </c>
+      <c r="D23" s="120">
+        <v>2.5</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B24" s="57" t="s">
+        <v>191</v>
+      </c>
+      <c r="C24" s="44" t="s">
+        <v>130</v>
+      </c>
+      <c r="D24" s="122">
+        <v>-0.04</v>
+      </c>
+      <c r="E24" s="59"/>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B26" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B27" s="147" t="s">
+        <v>190</v>
+      </c>
+      <c r="C27" s="147"/>
+      <c r="D27" s="147"/>
+      <c r="E27" s="147"/>
+    </row>
+    <row r="28" spans="2:5" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B28" s="146" t="s">
+        <v>189</v>
+      </c>
+      <c r="C28" s="146"/>
+      <c r="D28" s="146"/>
+      <c r="E28" s="146"/>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B4:E24">
+    <sortCondition ref="B4:B24"/>
+  </sortState>
+  <mergeCells count="3">
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="B27:E27"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADEA2BDB-C3E1-44CB-9C55-0D4DAE7C9E21}">
   <dimension ref="B1:J28"/>
   <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -3355,12 +3840,12 @@
       <c r="H1" s="17"/>
     </row>
     <row r="2" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B2" s="125" t="s">
+      <c r="B2" s="128" t="s">
         <v>160</v>
       </c>
-      <c r="C2" s="126"/>
-      <c r="D2" s="126"/>
-      <c r="E2" s="127"/>
+      <c r="C2" s="129"/>
+      <c r="D2" s="129"/>
+      <c r="E2" s="130"/>
       <c r="G2" s="39" t="s">
         <v>22</v>
       </c>
@@ -3638,20 +4123,20 @@
       </c>
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B23" s="144" t="s">
+      <c r="B23" s="147" t="s">
         <v>220</v>
       </c>
-      <c r="C23" s="144"/>
-      <c r="D23" s="144"/>
-      <c r="E23" s="144"/>
+      <c r="C23" s="147"/>
+      <c r="D23" s="147"/>
+      <c r="E23" s="147"/>
     </row>
     <row r="24" spans="2:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="143" t="s">
+      <c r="B24" s="146" t="s">
         <v>211</v>
       </c>
-      <c r="C24" s="143"/>
-      <c r="D24" s="143"/>
-      <c r="E24" s="143"/>
+      <c r="C24" s="146"/>
+      <c r="D24" s="146"/>
+      <c r="E24" s="146"/>
     </row>
     <row r="28" spans="2:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
@@ -3667,7 +4152,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBC421A3-3246-4411-B419-5D8153201591}">
   <dimension ref="B1:H19"/>
   <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -3681,12 +4166,12 @@
   <sheetData>
     <row r="1" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B2" s="125" t="s">
+      <c r="B2" s="128" t="s">
         <v>226</v>
       </c>
-      <c r="C2" s="126"/>
-      <c r="D2" s="126"/>
-      <c r="E2" s="127"/>
+      <c r="C2" s="129"/>
+      <c r="D2" s="129"/>
+      <c r="E2" s="130"/>
       <c r="G2" s="106" t="s">
         <v>22</v>
       </c>
@@ -3882,18 +4367,18 @@
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B18" s="144" t="s">
+      <c r="B18" s="147" t="s">
         <v>227</v>
       </c>
-      <c r="C18" s="144"/>
-      <c r="D18" s="144"/>
-      <c r="E18" s="144"/>
+      <c r="C18" s="147"/>
+      <c r="D18" s="147"/>
+      <c r="E18" s="147"/>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B19" s="143"/>
-      <c r="C19" s="143"/>
-      <c r="D19" s="143"/>
-      <c r="E19" s="143"/>
+      <c r="B19" s="146"/>
+      <c r="C19" s="146"/>
+      <c r="D19" s="146"/>
+      <c r="E19" s="146"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B4:E15">
@@ -3908,7 +4393,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{408C8F62-9799-4BD2-83D2-D7B5BA3D880C}">
   <dimension ref="B1:H12"/>
   <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -3925,12 +4410,12 @@
       <c r="H1" s="17"/>
     </row>
     <row r="2" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B2" s="125" t="s">
+      <c r="B2" s="128" t="s">
         <v>240</v>
       </c>
-      <c r="C2" s="126"/>
-      <c r="D2" s="126"/>
-      <c r="E2" s="127"/>
+      <c r="C2" s="129"/>
+      <c r="D2" s="129"/>
+      <c r="E2" s="130"/>
       <c r="G2" s="39" t="s">
         <v>22</v>
       </c>
@@ -4052,12 +4537,12 @@
       </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B12" s="144" t="s">
+      <c r="B12" s="147" t="s">
         <v>239</v>
       </c>
-      <c r="C12" s="144"/>
-      <c r="D12" s="144"/>
-      <c r="E12" s="144"/>
+      <c r="C12" s="147"/>
+      <c r="D12" s="147"/>
+      <c r="E12" s="147"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4068,7 +4553,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE56C769-9962-4024-9DC3-A48D7248A933}">
   <dimension ref="A1:N54"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -4092,20 +4577,20 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="E2" s="145" t="s">
+      <c r="E2" s="148" t="s">
         <v>133</v>
       </c>
-      <c r="F2" s="145"/>
-      <c r="G2" s="145"/>
-      <c r="H2" s="145"/>
-      <c r="I2" s="145"/>
-      <c r="J2" s="145"/>
-      <c r="K2" s="146" t="s">
+      <c r="F2" s="148"/>
+      <c r="G2" s="148"/>
+      <c r="H2" s="148"/>
+      <c r="I2" s="148"/>
+      <c r="J2" s="148"/>
+      <c r="K2" s="149" t="s">
         <v>134</v>
       </c>
-      <c r="L2" s="146"/>
-      <c r="M2" s="146"/>
-      <c r="N2" s="146"/>
+      <c r="L2" s="149"/>
+      <c r="M2" s="149"/>
+      <c r="N2" s="149"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="71" t="s">
@@ -4117,12 +4602,12 @@
       <c r="C3" s="71" t="s">
         <v>136</v>
       </c>
-      <c r="E3" s="145"/>
-      <c r="F3" s="145"/>
-      <c r="G3" s="145"/>
-      <c r="H3" s="145"/>
-      <c r="I3" s="145"/>
-      <c r="J3" s="145"/>
+      <c r="E3" s="148"/>
+      <c r="F3" s="148"/>
+      <c r="G3" s="148"/>
+      <c r="H3" s="148"/>
+      <c r="I3" s="148"/>
+      <c r="J3" s="148"/>
       <c r="K3" s="72" t="s">
         <v>137</v>
       </c>
@@ -5092,7 +5577,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F08D047-F0FC-4BFB-97BC-1391B65AB4E5}">
   <dimension ref="A1:N69"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -5116,20 +5601,20 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="E2" s="145" t="s">
+      <c r="E2" s="148" t="s">
         <v>133</v>
       </c>
-      <c r="F2" s="145"/>
-      <c r="G2" s="145"/>
-      <c r="H2" s="145"/>
-      <c r="I2" s="145"/>
-      <c r="J2" s="145"/>
-      <c r="K2" s="146" t="s">
+      <c r="F2" s="148"/>
+      <c r="G2" s="148"/>
+      <c r="H2" s="148"/>
+      <c r="I2" s="148"/>
+      <c r="J2" s="148"/>
+      <c r="K2" s="149" t="s">
         <v>134</v>
       </c>
-      <c r="L2" s="146"/>
-      <c r="M2" s="146"/>
-      <c r="N2" s="146"/>
+      <c r="L2" s="149"/>
+      <c r="M2" s="149"/>
+      <c r="N2" s="149"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="71" t="s">
@@ -5141,12 +5626,12 @@
       <c r="C3" s="71" t="s">
         <v>136</v>
       </c>
-      <c r="E3" s="145"/>
-      <c r="F3" s="145"/>
-      <c r="G3" s="145"/>
-      <c r="H3" s="145"/>
-      <c r="I3" s="145"/>
-      <c r="J3" s="145"/>
+      <c r="E3" s="148"/>
+      <c r="F3" s="148"/>
+      <c r="G3" s="148"/>
+      <c r="H3" s="148"/>
+      <c r="I3" s="148"/>
+      <c r="J3" s="148"/>
       <c r="K3" s="72" t="s">
         <v>137</v>
       </c>
@@ -6500,7 +6985,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72A54061-D842-48D6-BC83-5179935F2CE7}">
   <dimension ref="A1:J34"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -6523,17 +7008,17 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="D2" s="145" t="s">
+      <c r="D2" s="148" t="s">
         <v>133</v>
       </c>
-      <c r="E2" s="145"/>
-      <c r="F2" s="145"/>
-      <c r="G2" s="146" t="s">
+      <c r="E2" s="148"/>
+      <c r="F2" s="148"/>
+      <c r="G2" s="149" t="s">
         <v>134</v>
       </c>
-      <c r="H2" s="146"/>
-      <c r="I2" s="146"/>
-      <c r="J2" s="146"/>
+      <c r="H2" s="149"/>
+      <c r="I2" s="149"/>
+      <c r="J2" s="149"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="71" t="s">
@@ -6542,9 +7027,9 @@
       <c r="B3" s="71" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="145"/>
-      <c r="E3" s="145"/>
-      <c r="F3" s="145"/>
+      <c r="D3" s="148"/>
+      <c r="E3" s="148"/>
+      <c r="F3" s="148"/>
       <c r="G3" s="72" t="s">
         <v>137</v>
       </c>
@@ -6891,7 +7376,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CD52CBF-D6A2-4A23-B04A-BA9A88472FF0}">
   <dimension ref="A1:N56"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -6914,20 +7399,20 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="D2" s="145" t="s">
+      <c r="D2" s="148" t="s">
         <v>133</v>
       </c>
-      <c r="E2" s="145"/>
-      <c r="F2" s="145"/>
-      <c r="G2" s="145"/>
-      <c r="H2" s="145"/>
-      <c r="I2" s="145"/>
-      <c r="J2" s="146" t="s">
+      <c r="E2" s="148"/>
+      <c r="F2" s="148"/>
+      <c r="G2" s="148"/>
+      <c r="H2" s="148"/>
+      <c r="I2" s="148"/>
+      <c r="J2" s="149" t="s">
         <v>134</v>
       </c>
-      <c r="K2" s="146"/>
-      <c r="L2" s="146"/>
-      <c r="M2" s="146"/>
+      <c r="K2" s="149"/>
+      <c r="L2" s="149"/>
+      <c r="M2" s="149"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="71" t="s">
@@ -6936,12 +7421,12 @@
       <c r="B3" s="71" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="145"/>
-      <c r="E3" s="145"/>
-      <c r="F3" s="145"/>
-      <c r="G3" s="145"/>
-      <c r="H3" s="145"/>
-      <c r="I3" s="145"/>
+      <c r="D3" s="148"/>
+      <c r="E3" s="148"/>
+      <c r="F3" s="148"/>
+      <c r="G3" s="148"/>
+      <c r="H3" s="148"/>
+      <c r="I3" s="148"/>
       <c r="J3" s="72" t="s">
         <v>137</v>
       </c>
@@ -7733,7 +8218,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C39FC881-A3CB-406E-9F4D-21C24E806799}">
   <dimension ref="A1:K34"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -7756,17 +8241,17 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="D2" s="145" t="s">
+      <c r="D2" s="148" t="s">
         <v>133</v>
       </c>
-      <c r="E2" s="145"/>
-      <c r="F2" s="145"/>
-      <c r="G2" s="146" t="s">
+      <c r="E2" s="148"/>
+      <c r="F2" s="148"/>
+      <c r="G2" s="149" t="s">
         <v>134</v>
       </c>
-      <c r="H2" s="146"/>
-      <c r="I2" s="146"/>
-      <c r="J2" s="146"/>
+      <c r="H2" s="149"/>
+      <c r="I2" s="149"/>
+      <c r="J2" s="149"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="71" t="s">
@@ -7775,9 +8260,9 @@
       <c r="B3" s="71" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="145"/>
-      <c r="E3" s="145"/>
-      <c r="F3" s="145"/>
+      <c r="D3" s="148"/>
+      <c r="E3" s="148"/>
+      <c r="F3" s="148"/>
       <c r="G3" s="72" t="s">
         <v>137</v>
       </c>
@@ -8131,1009 +8616,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE247F88-6DDE-433E-81AC-06E8044E24FC}">
-  <dimension ref="B1:H10"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.58203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.83203125" customWidth="1"/>
-    <col min="5" max="5" width="15.75" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-    </row>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B2" s="128" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="131"/>
-      <c r="D2" s="129"/>
-      <c r="E2" s="130"/>
-      <c r="G2" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H2" s="8">
-        <v>50.688999199999998</v>
-      </c>
-    </row>
-    <row r="3" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="21" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="62"/>
-      <c r="D3" s="18" t="s">
-        <v>4</v>
-      </c>
-      <c r="E3" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="G3" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="3">
-        <v>-63.2494011</v>
-      </c>
-    </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B4" s="23" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="63" t="s">
-        <v>108</v>
-      </c>
-      <c r="D4" s="19">
-        <v>1.5</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="5" spans="2:8" ht="31" x14ac:dyDescent="0.35">
-      <c r="B5" s="24" t="s">
-        <v>2</v>
-      </c>
-      <c r="C5" s="66" t="s">
-        <v>109</v>
-      </c>
-      <c r="D5" s="20">
-        <v>2</v>
-      </c>
-      <c r="E5" s="1"/>
-    </row>
-    <row r="6" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="25" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="65"/>
-      <c r="D6" s="26">
-        <v>2</v>
-      </c>
-      <c r="E6" s="12"/>
-    </row>
-    <row r="7" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B8" s="128" t="s">
-        <v>47</v>
-      </c>
-      <c r="C8" s="129"/>
-      <c r="D8" s="129"/>
-      <c r="E8" s="130"/>
-    </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B9" s="21"/>
-      <c r="C9" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="D9" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="E9" s="22" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="10" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B10" s="25" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" s="26">
-        <v>85</v>
-      </c>
-      <c r="D10" s="26">
-        <v>-10</v>
-      </c>
-      <c r="E10" s="12">
-        <v>-10</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B8:E8"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53111C9A-58C1-40C7-9383-CFE5F1F570E0}">
-  <dimension ref="B1:G57"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="2" max="2" width="10.08203125" customWidth="1"/>
-    <col min="3" max="3" width="24.58203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.58203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.08203125" customWidth="1"/>
-    <col min="7" max="7" width="9.58203125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:7" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-    </row>
-    <row r="2" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B2" s="128" t="s">
-        <v>48</v>
-      </c>
-      <c r="C2" s="129"/>
-      <c r="D2" s="130"/>
-      <c r="F2" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G2" s="8">
-        <v>50.689498899999997</v>
-      </c>
-    </row>
-    <row r="3" spans="2:7" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="21" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="18" t="s">
-        <v>107</v>
-      </c>
-      <c r="D3" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="F3" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="G3" s="3">
-        <v>-63.249698600000002</v>
-      </c>
-    </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B4" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D4" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B5" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D5" s="11">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B6" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D6" s="1">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B7" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D7" s="11">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B8" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D8" s="1">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B9" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D9" s="11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B10" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D10" s="1">
-        <v>1.4</v>
-      </c>
-    </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B11" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D11" s="1">
-        <v>1.8</v>
-      </c>
-    </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B12" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D12" s="1">
-        <v>2.2000000000000002</v>
-      </c>
-    </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B13" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D13" s="11">
-        <v>2.6</v>
-      </c>
-    </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B14" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C14" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D14" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B15" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C15" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D15" s="11">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B16" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D16" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B17" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C17" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D17" s="11">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B18" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C18" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D18" s="1">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B19" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C19" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D19" s="11">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B20" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C20" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D20" s="1">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B21" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C21" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D21" s="11">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B22" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C22" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D22" s="1">
-        <v>12.5</v>
-      </c>
-    </row>
-    <row r="23" spans="2:7" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B23" s="25" t="s">
-        <v>18</v>
-      </c>
-      <c r="C23" s="26" t="s">
-        <v>121</v>
-      </c>
-      <c r="D23" s="12">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="24" spans="2:7" ht="16" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B25" s="128" t="s">
-        <v>16</v>
-      </c>
-      <c r="C25" s="129"/>
-      <c r="D25" s="130"/>
-      <c r="F25" s="39" t="s">
-        <v>22</v>
-      </c>
-      <c r="G25" s="40">
-        <v>50.6753006</v>
-      </c>
-    </row>
-    <row r="26" spans="2:7" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B26" s="21" t="s">
-        <v>0</v>
-      </c>
-      <c r="C26" s="18" t="s">
-        <v>107</v>
-      </c>
-      <c r="D26" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="F26" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="G26" s="3">
-        <v>-63.2527008</v>
-      </c>
-    </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B27" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C27" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D27" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B28" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C28" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D28" s="11">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B29" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C29" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D29" s="1">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B30" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C30" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D30" s="11">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B31" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C31" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D31" s="1">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B32" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C32" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D32" s="11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B33" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C33" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D33" s="1">
-        <v>1.4</v>
-      </c>
-    </row>
-    <row r="34" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B34" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C34" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D34" s="1">
-        <v>1.8</v>
-      </c>
-    </row>
-    <row r="35" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B35" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C35" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D35" s="1">
-        <v>2.2000000000000002</v>
-      </c>
-    </row>
-    <row r="36" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B36" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C36" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D36" s="11">
-        <v>2.6</v>
-      </c>
-    </row>
-    <row r="37" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B37" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C37" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D37" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="38" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B38" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C38" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D38" s="11">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="39" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B39" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C39" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D39" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="40" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B40" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C40" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D40" s="11">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="41" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B41" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C41" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D41" s="1">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="42" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B42" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C42" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D42" s="11">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="43" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B43" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C43" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D43" s="1">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="44" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B44" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C44" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D44" s="11">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="45" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B45" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C45" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D45" s="1">
-        <v>12.5</v>
-      </c>
-    </row>
-    <row r="46" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B46" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C46" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D46" s="11">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="47" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B47" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C47" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D47" s="1">
-        <v>17.5</v>
-      </c>
-    </row>
-    <row r="48" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B48" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C48" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D48" s="11">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="49" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B49" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C49" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D49" s="1">
-        <v>22.5</v>
-      </c>
-    </row>
-    <row r="50" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B50" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C50" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D50" s="11">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="51" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B51" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C51" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D51" s="1">
-        <v>27.5</v>
-      </c>
-    </row>
-    <row r="52" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B52" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C52" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D52" s="11">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="53" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B53" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C53" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D53" s="1">
-        <v>32.5</v>
-      </c>
-    </row>
-    <row r="54" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B54" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C54" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="D54" s="11">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="55" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B55" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C55" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D55" s="1">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="56" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B56" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C56" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="D56" s="11">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="57" spans="2:4" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B57" s="30" t="s">
-        <v>18</v>
-      </c>
-      <c r="C57" s="44" t="s">
-        <v>121</v>
-      </c>
-      <c r="D57" s="2">
-        <v>70</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B25:D25"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B1D1867-B0BA-4CF9-B964-CDDBB5D9DD8C}">
-  <dimension ref="B1:H18"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.75" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.08203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.58203125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B2" s="125" t="s">
-        <v>39</v>
-      </c>
-      <c r="C2" s="126"/>
-      <c r="D2" s="126"/>
-      <c r="E2" s="127"/>
-      <c r="G2" s="29" t="s">
-        <v>22</v>
-      </c>
-      <c r="H2" s="15">
-        <v>50.861454700000003</v>
-      </c>
-    </row>
-    <row r="3" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="21" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="18" t="s">
-        <v>107</v>
-      </c>
-      <c r="D3" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="E3" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="G3" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="2">
-        <v>-63.389840900000003</v>
-      </c>
-    </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B4" s="23" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="19" t="s">
-        <v>108</v>
-      </c>
-      <c r="D4" s="19">
-        <v>0.8</v>
-      </c>
-      <c r="E4" s="11"/>
-    </row>
-    <row r="5" spans="2:8" ht="31" x14ac:dyDescent="0.35">
-      <c r="B5" s="24" t="s">
-        <v>2</v>
-      </c>
-      <c r="C5" s="64" t="s">
-        <v>109</v>
-      </c>
-      <c r="D5" s="20">
-        <v>4.3</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B6" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19">
-        <v>4.3</v>
-      </c>
-      <c r="E6" s="11"/>
-    </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B7" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>110</v>
-      </c>
-      <c r="D7" s="20">
-        <v>4.3</v>
-      </c>
-      <c r="E7" s="1"/>
-    </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B8" s="23" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="19" t="s">
-        <v>111</v>
-      </c>
-      <c r="D8" s="19">
-        <v>3.9</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B9" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>112</v>
-      </c>
-      <c r="D9" s="20">
-        <v>0.8</v>
-      </c>
-      <c r="E9" s="27"/>
-    </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B10" s="23" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" s="19" t="s">
-        <v>113</v>
-      </c>
-      <c r="D10" s="19">
-        <v>2</v>
-      </c>
-      <c r="E10" s="11"/>
-    </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B11" s="24" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="20" t="s">
-        <v>114</v>
-      </c>
-      <c r="D11" s="20">
-        <v>1.2</v>
-      </c>
-      <c r="E11" s="1"/>
-    </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B12" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="C12" s="19" t="s">
-        <v>115</v>
-      </c>
-      <c r="D12" s="19">
-        <v>1</v>
-      </c>
-      <c r="E12" s="11"/>
-    </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B13" s="147" t="s">
-        <v>243</v>
-      </c>
-      <c r="C13" s="148" t="s">
-        <v>244</v>
-      </c>
-      <c r="D13" s="148">
-        <v>1.2</v>
-      </c>
-      <c r="E13" s="149"/>
-    </row>
-    <row r="14" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B14" s="25" t="s">
-        <v>83</v>
-      </c>
-      <c r="C14" s="26" t="s">
-        <v>116</v>
-      </c>
-      <c r="D14" s="26">
-        <v>1</v>
-      </c>
-      <c r="E14" s="12" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="15" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B16" s="128" t="s">
-        <v>33</v>
-      </c>
-      <c r="C16" s="129"/>
-      <c r="D16" s="129"/>
-      <c r="E16" s="130"/>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B17" s="21"/>
-      <c r="C17" s="18" t="s">
-        <v>34</v>
-      </c>
-      <c r="D17" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="E17" s="22" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="18" spans="2:5" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B18" s="25" t="s">
-        <v>5</v>
-      </c>
-      <c r="C18" s="26">
-        <v>-37.5</v>
-      </c>
-      <c r="D18" s="26">
-        <v>5.5</v>
-      </c>
-      <c r="E18" s="12">
-        <v>7</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B16:E16"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8BF41A8-026E-451A-9D63-213454538E4C}">
   <dimension ref="B1:G24"/>
   <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -9144,11 +8626,11 @@
   <sheetData>
     <row r="1" spans="2:7" ht="16" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B2" s="128" t="s">
+      <c r="B2" s="131" t="s">
         <v>49</v>
       </c>
-      <c r="C2" s="129"/>
-      <c r="D2" s="130"/>
+      <c r="C2" s="132"/>
+      <c r="D2" s="133"/>
       <c r="F2" s="39" t="s">
         <v>22</v>
       </c>
@@ -9412,7 +8894,102 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CBC5DDE-AFB1-4D48-9B4E-CD429852D58B}">
+  <dimension ref="B1:H6"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="15.58203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.75" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="43" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="2" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B2" s="128" t="s">
+        <v>245</v>
+      </c>
+      <c r="C2" s="129"/>
+      <c r="D2" s="129"/>
+      <c r="E2" s="130"/>
+      <c r="G2" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="15">
+        <v>50.901774000000003</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B3" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="G3" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="2">
+        <v>-63.404361999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B4" s="23" t="s">
+        <v>246</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>248</v>
+      </c>
+      <c r="D4" s="151">
+        <v>0.64</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B5" s="24" t="s">
+        <v>247</v>
+      </c>
+      <c r="C5" s="64" t="s">
+        <v>249</v>
+      </c>
+      <c r="D5" s="152">
+        <v>2.7229999999999999</v>
+      </c>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" spans="2:8" ht="31.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B6" s="25" t="s">
+        <v>250</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>244</v>
+      </c>
+      <c r="D6" s="153" t="s">
+        <v>252</v>
+      </c>
+      <c r="E6" s="150" t="s">
+        <v>253</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:E2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DE59413-D9F3-44A1-88DC-A59245E9D9B8}">
   <dimension ref="B1:J27"/>
   <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -9428,12 +9005,12 @@
   <sheetData>
     <row r="1" spans="2:10" ht="16" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B2" s="125" t="s">
+      <c r="B2" s="128" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="126"/>
-      <c r="D2" s="126"/>
-      <c r="E2" s="127"/>
+      <c r="C2" s="129"/>
+      <c r="D2" s="129"/>
+      <c r="E2" s="130"/>
       <c r="G2" s="39" t="s">
         <v>22</v>
       </c>
@@ -9486,12 +9063,12 @@
       <c r="E5" s="38" t="s">
         <v>93</v>
       </c>
-      <c r="G5" s="128" t="s">
+      <c r="G5" s="131" t="s">
         <v>33</v>
       </c>
-      <c r="H5" s="129"/>
-      <c r="I5" s="129"/>
-      <c r="J5" s="130"/>
+      <c r="H5" s="132"/>
+      <c r="I5" s="132"/>
+      <c r="J5" s="133"/>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B6" s="54" t="s">
@@ -9844,7 +9421,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D03A187-FF98-4B1B-892D-A571F19F5DA5}">
   <dimension ref="A1:E44"/>
   <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -9872,10 +9449,10 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="16" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="132" t="s">
+      <c r="A2" s="135" t="s">
         <v>78</v>
       </c>
-      <c r="B2" s="136" t="s">
+      <c r="B2" s="139" t="s">
         <v>72</v>
       </c>
       <c r="C2" s="49" t="s">
@@ -9889,8 +9466,8 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="133"/>
-      <c r="B3" s="137"/>
+      <c r="A3" s="136"/>
+      <c r="B3" s="140"/>
       <c r="C3" s="45" t="s">
         <v>55</v>
       </c>
@@ -9902,8 +9479,8 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" s="133"/>
-      <c r="B4" s="138" t="s">
+      <c r="A4" s="136"/>
+      <c r="B4" s="141" t="s">
         <v>69</v>
       </c>
       <c r="C4" s="43" t="s">
@@ -9917,8 +9494,8 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="133"/>
-      <c r="B5" s="139"/>
+      <c r="A5" s="136"/>
+      <c r="B5" s="142"/>
       <c r="C5" s="41" t="s">
         <v>62</v>
       </c>
@@ -9930,8 +9507,8 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="133"/>
-      <c r="B6" s="139"/>
+      <c r="A6" s="136"/>
+      <c r="B6" s="142"/>
       <c r="C6" s="41" t="s">
         <v>60</v>
       </c>
@@ -9943,8 +9520,8 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" s="133"/>
-      <c r="B7" s="139"/>
+      <c r="A7" s="136"/>
+      <c r="B7" s="142"/>
       <c r="C7" s="41" t="s">
         <v>55</v>
       </c>
@@ -9956,8 +9533,8 @@
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" s="133"/>
-      <c r="B8" s="139"/>
+      <c r="A8" s="136"/>
+      <c r="B8" s="142"/>
       <c r="C8" s="41" t="s">
         <v>54</v>
       </c>
@@ -9969,8 +9546,8 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="133"/>
-      <c r="B9" s="137"/>
+      <c r="A9" s="136"/>
+      <c r="B9" s="140"/>
       <c r="C9" s="45" t="s">
         <v>52</v>
       </c>
@@ -9982,8 +9559,8 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" s="133"/>
-      <c r="B10" s="138" t="s">
+      <c r="A10" s="136"/>
+      <c r="B10" s="141" t="s">
         <v>67</v>
       </c>
       <c r="C10" s="43" t="s">
@@ -9997,8 +9574,8 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A11" s="133"/>
-      <c r="B11" s="139"/>
+      <c r="A11" s="136"/>
+      <c r="B11" s="142"/>
       <c r="C11" s="41" t="s">
         <v>62</v>
       </c>
@@ -10010,8 +9587,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" s="133"/>
-      <c r="B12" s="139"/>
+      <c r="A12" s="136"/>
+      <c r="B12" s="142"/>
       <c r="C12" s="41" t="s">
         <v>60</v>
       </c>
@@ -10023,8 +9600,8 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13" s="133"/>
-      <c r="B13" s="139"/>
+      <c r="A13" s="136"/>
+      <c r="B13" s="142"/>
       <c r="C13" s="41" t="s">
         <v>55</v>
       </c>
@@ -10036,8 +9613,8 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14" s="133"/>
-      <c r="B14" s="139"/>
+      <c r="A14" s="136"/>
+      <c r="B14" s="142"/>
       <c r="C14" s="41" t="s">
         <v>54</v>
       </c>
@@ -10049,8 +9626,8 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="133"/>
-      <c r="B15" s="137"/>
+      <c r="A15" s="136"/>
+      <c r="B15" s="140"/>
       <c r="C15" s="45" t="s">
         <v>52</v>
       </c>
@@ -10062,8 +9639,8 @@
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A16" s="133"/>
-      <c r="B16" s="138" t="s">
+      <c r="A16" s="136"/>
+      <c r="B16" s="141" t="s">
         <v>65</v>
       </c>
       <c r="C16" s="43" t="s">
@@ -10077,8 +9654,8 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A17" s="133"/>
-      <c r="B17" s="139"/>
+      <c r="A17" s="136"/>
+      <c r="B17" s="142"/>
       <c r="C17" s="41" t="s">
         <v>62</v>
       </c>
@@ -10090,8 +9667,8 @@
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" s="133"/>
-      <c r="B18" s="139"/>
+      <c r="A18" s="136"/>
+      <c r="B18" s="142"/>
       <c r="C18" s="41" t="s">
         <v>60</v>
       </c>
@@ -10103,8 +9680,8 @@
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A19" s="133"/>
-      <c r="B19" s="139"/>
+      <c r="A19" s="136"/>
+      <c r="B19" s="142"/>
       <c r="C19" s="41" t="s">
         <v>55</v>
       </c>
@@ -10116,8 +9693,8 @@
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" s="133"/>
-      <c r="B20" s="139"/>
+      <c r="A20" s="136"/>
+      <c r="B20" s="142"/>
       <c r="C20" s="41" t="s">
         <v>54</v>
       </c>
@@ -10129,8 +9706,8 @@
       </c>
     </row>
     <row r="21" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="134"/>
-      <c r="B21" s="140"/>
+      <c r="A21" s="137"/>
+      <c r="B21" s="143"/>
       <c r="C21" s="47" t="s">
         <v>52</v>
       </c>
@@ -10142,10 +9719,10 @@
       </c>
     </row>
     <row r="22" spans="1:5" ht="16" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="135" t="s">
+      <c r="A22" s="138" t="s">
         <v>73</v>
       </c>
-      <c r="B22" s="138" t="s">
+      <c r="B22" s="141" t="s">
         <v>72</v>
       </c>
       <c r="C22" s="43" t="s">
@@ -10159,8 +9736,8 @@
       </c>
     </row>
     <row r="23" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="133"/>
-      <c r="B23" s="137"/>
+      <c r="A23" s="136"/>
+      <c r="B23" s="140"/>
       <c r="C23" s="45" t="s">
         <v>55</v>
       </c>
@@ -10172,8 +9749,8 @@
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A24" s="133"/>
-      <c r="B24" s="138" t="s">
+      <c r="A24" s="136"/>
+      <c r="B24" s="141" t="s">
         <v>69</v>
       </c>
       <c r="C24" s="43" t="s">
@@ -10187,8 +9764,8 @@
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A25" s="133"/>
-      <c r="B25" s="139"/>
+      <c r="A25" s="136"/>
+      <c r="B25" s="142"/>
       <c r="C25" s="41" t="s">
         <v>62</v>
       </c>
@@ -10200,8 +9777,8 @@
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A26" s="133"/>
-      <c r="B26" s="139"/>
+      <c r="A26" s="136"/>
+      <c r="B26" s="142"/>
       <c r="C26" s="41" t="s">
         <v>60</v>
       </c>
@@ -10213,8 +9790,8 @@
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A27" s="133"/>
-      <c r="B27" s="139"/>
+      <c r="A27" s="136"/>
+      <c r="B27" s="142"/>
       <c r="C27" s="41" t="s">
         <v>57</v>
       </c>
@@ -10226,8 +9803,8 @@
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A28" s="133"/>
-      <c r="B28" s="139"/>
+      <c r="A28" s="136"/>
+      <c r="B28" s="142"/>
       <c r="C28" s="41" t="s">
         <v>55</v>
       </c>
@@ -10239,8 +9816,8 @@
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A29" s="133"/>
-      <c r="B29" s="139"/>
+      <c r="A29" s="136"/>
+      <c r="B29" s="142"/>
       <c r="C29" s="41" t="s">
         <v>54</v>
       </c>
@@ -10252,8 +9829,8 @@
       </c>
     </row>
     <row r="30" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A30" s="133"/>
-      <c r="B30" s="137"/>
+      <c r="A30" s="136"/>
+      <c r="B30" s="140"/>
       <c r="C30" s="45" t="s">
         <v>52</v>
       </c>
@@ -10265,8 +9842,8 @@
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A31" s="133"/>
-      <c r="B31" s="138" t="s">
+      <c r="A31" s="136"/>
+      <c r="B31" s="141" t="s">
         <v>67</v>
       </c>
       <c r="C31" s="43" t="s">
@@ -10280,8 +9857,8 @@
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A32" s="133"/>
-      <c r="B32" s="139"/>
+      <c r="A32" s="136"/>
+      <c r="B32" s="142"/>
       <c r="C32" s="41" t="s">
         <v>62</v>
       </c>
@@ -10293,8 +9870,8 @@
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A33" s="133"/>
-      <c r="B33" s="139"/>
+      <c r="A33" s="136"/>
+      <c r="B33" s="142"/>
       <c r="C33" s="41" t="s">
         <v>60</v>
       </c>
@@ -10306,8 +9883,8 @@
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A34" s="133"/>
-      <c r="B34" s="139"/>
+      <c r="A34" s="136"/>
+      <c r="B34" s="142"/>
       <c r="C34" s="41" t="s">
         <v>57</v>
       </c>
@@ -10319,8 +9896,8 @@
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A35" s="133"/>
-      <c r="B35" s="139"/>
+      <c r="A35" s="136"/>
+      <c r="B35" s="142"/>
       <c r="C35" s="41" t="s">
         <v>55</v>
       </c>
@@ -10332,8 +9909,8 @@
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A36" s="133"/>
-      <c r="B36" s="139"/>
+      <c r="A36" s="136"/>
+      <c r="B36" s="142"/>
       <c r="C36" s="41" t="s">
         <v>54</v>
       </c>
@@ -10345,8 +9922,8 @@
       </c>
     </row>
     <row r="37" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A37" s="133"/>
-      <c r="B37" s="137"/>
+      <c r="A37" s="136"/>
+      <c r="B37" s="140"/>
       <c r="C37" s="45" t="s">
         <v>52</v>
       </c>
@@ -10358,8 +9935,8 @@
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A38" s="133"/>
-      <c r="B38" s="138" t="s">
+      <c r="A38" s="136"/>
+      <c r="B38" s="141" t="s">
         <v>65</v>
       </c>
       <c r="C38" s="43" t="s">
@@ -10373,8 +9950,8 @@
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A39" s="133"/>
-      <c r="B39" s="139"/>
+      <c r="A39" s="136"/>
+      <c r="B39" s="142"/>
       <c r="C39" s="41" t="s">
         <v>62</v>
       </c>
@@ -10386,8 +9963,8 @@
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A40" s="133"/>
-      <c r="B40" s="139"/>
+      <c r="A40" s="136"/>
+      <c r="B40" s="142"/>
       <c r="C40" s="41" t="s">
         <v>60</v>
       </c>
@@ -10399,8 +9976,8 @@
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A41" s="133"/>
-      <c r="B41" s="139"/>
+      <c r="A41" s="136"/>
+      <c r="B41" s="142"/>
       <c r="C41" s="41" t="s">
         <v>57</v>
       </c>
@@ -10412,8 +9989,8 @@
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A42" s="133"/>
-      <c r="B42" s="139"/>
+      <c r="A42" s="136"/>
+      <c r="B42" s="142"/>
       <c r="C42" s="41" t="s">
         <v>55</v>
       </c>
@@ -10425,8 +10002,8 @@
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A43" s="133"/>
-      <c r="B43" s="139"/>
+      <c r="A43" s="136"/>
+      <c r="B43" s="142"/>
       <c r="C43" s="41" t="s">
         <v>54</v>
       </c>
@@ -10438,8 +10015,8 @@
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A44" s="133"/>
-      <c r="B44" s="139"/>
+      <c r="A44" s="136"/>
+      <c r="B44" s="142"/>
       <c r="C44" s="41" t="s">
         <v>52</v>
       </c>
@@ -10467,7 +10044,998 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE247F88-6DDE-433E-81AC-06E8044E24FC}">
+  <dimension ref="B1:H10"/>
+  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.58203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.75" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+    </row>
+    <row r="2" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B2" s="131" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="134"/>
+      <c r="D2" s="132"/>
+      <c r="E2" s="133"/>
+      <c r="G2" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="8">
+        <v>50.688999199999998</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B3" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="62"/>
+      <c r="D3" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="G3" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="3">
+        <v>-63.2494011</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B4" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="63" t="s">
+        <v>108</v>
+      </c>
+      <c r="D4" s="19">
+        <v>1.5</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" ht="31" x14ac:dyDescent="0.35">
+      <c r="B5" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="66" t="s">
+        <v>109</v>
+      </c>
+      <c r="D5" s="20">
+        <v>2</v>
+      </c>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B6" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="65"/>
+      <c r="D6" s="26">
+        <v>2</v>
+      </c>
+      <c r="E6" s="12"/>
+    </row>
+    <row r="7" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B8" s="131" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" s="132"/>
+      <c r="D8" s="132"/>
+      <c r="E8" s="133"/>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B9" s="21"/>
+      <c r="C9" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="E9" s="22" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B10" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="26">
+        <v>85</v>
+      </c>
+      <c r="D10" s="26">
+        <v>-10</v>
+      </c>
+      <c r="E10" s="12">
+        <v>-10</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B8:E8"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE44D4E6-1DC8-5846-9613-DEB0E908B686}">
+  <dimension ref="B1:J16"/>
+  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="17.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.75" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.75" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+    <col min="7" max="7" width="11.25" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.33203125" customWidth="1"/>
+    <col min="9" max="9" width="25.33203125" customWidth="1"/>
+    <col min="10" max="10" width="20.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:10" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+    </row>
+    <row r="2" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B2" s="128" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="129"/>
+      <c r="D2" s="129"/>
+      <c r="E2" s="130"/>
+      <c r="G2" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="8">
+        <v>50.653801000000001</v>
+      </c>
+    </row>
+    <row r="3" spans="2:10" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B3" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="G3" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="3">
+        <v>-63.259498600000001</v>
+      </c>
+    </row>
+    <row r="4" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B4" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="D4" s="19">
+        <v>8</v>
+      </c>
+      <c r="E4" s="11"/>
+    </row>
+    <row r="5" spans="2:10" ht="31" x14ac:dyDescent="0.35">
+      <c r="B5" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="64" t="s">
+        <v>117</v>
+      </c>
+      <c r="D5" s="20">
+        <v>7.25</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B6" s="23" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="19"/>
+      <c r="D6" s="19">
+        <v>7.25</v>
+      </c>
+      <c r="E6" s="11"/>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B7" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>110</v>
+      </c>
+      <c r="D7" s="20">
+        <v>7.25</v>
+      </c>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B8" s="23" t="s">
+        <v>92</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>242</v>
+      </c>
+      <c r="D8" s="19">
+        <v>2.5</v>
+      </c>
+      <c r="E8" s="60" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B9" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="D9" s="20">
+        <v>6.3</v>
+      </c>
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B10" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="D10" s="19">
+        <v>5.2</v>
+      </c>
+      <c r="E10" s="61" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B11" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>113</v>
+      </c>
+      <c r="D11" s="20">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" spans="2:10" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="26" t="s">
+        <v>115</v>
+      </c>
+      <c r="D12" s="26">
+        <v>0.9</v>
+      </c>
+      <c r="E12" s="12"/>
+    </row>
+    <row r="13" spans="2:10" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="G13" s="28"/>
+      <c r="H13" s="28"/>
+      <c r="I13" s="28"/>
+      <c r="J13" s="28"/>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B14" s="131" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" s="132"/>
+      <c r="D14" s="132"/>
+      <c r="E14" s="133"/>
+    </row>
+    <row r="15" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B15" s="21"/>
+      <c r="C15" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="E15" s="22" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="16" spans="2:10" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B16" s="25" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="26">
+        <v>26</v>
+      </c>
+      <c r="D16" s="26">
+        <v>-13.6</v>
+      </c>
+      <c r="E16" s="12">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B14:E14"/>
+  </mergeCells>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53111C9A-58C1-40C7-9383-CFE5F1F570E0}">
+  <dimension ref="B1:G57"/>
+  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="10.08203125" customWidth="1"/>
+    <col min="3" max="3" width="24.58203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.58203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.08203125" customWidth="1"/>
+    <col min="7" max="7" width="9.58203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:7" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+    </row>
+    <row r="2" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B2" s="131" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="132"/>
+      <c r="D2" s="133"/>
+      <c r="F2" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G2" s="8">
+        <v>50.689498899999997</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B3" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="D3" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="3">
+        <v>-63.249698600000002</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B4" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D4" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B5" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D5" s="11">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B6" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D6" s="1">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B7" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D7" s="11">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B8" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D8" s="1">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B9" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D9" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B10" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D10" s="1">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B11" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D11" s="1">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B12" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D12" s="1">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B13" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D13" s="11">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B14" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D14" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B15" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D15" s="11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B16" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D16" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B17" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D17" s="11">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B18" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D18" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B19" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D19" s="11">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B20" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C20" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D20" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B21" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D21" s="11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B22" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D22" s="1">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B23" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="26" t="s">
+        <v>121</v>
+      </c>
+      <c r="D23" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" ht="16" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B25" s="131" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="132"/>
+      <c r="D25" s="133"/>
+      <c r="F25" s="39" t="s">
+        <v>22</v>
+      </c>
+      <c r="G25" s="40">
+        <v>50.6753006</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B26" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="D26" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="F26" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="G26" s="3">
+        <v>-63.2527008</v>
+      </c>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B27" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C27" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D27" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B28" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C28" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D28" s="11">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B29" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C29" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D29" s="1">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B30" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C30" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D30" s="11">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="31" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B31" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C31" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D31" s="1">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B32" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C32" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D32" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B33" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C33" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D33" s="1">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="34" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B34" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C34" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D34" s="1">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="35" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B35" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C35" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D35" s="1">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="36" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B36" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C36" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D36" s="11">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="37" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B37" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C37" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D37" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B38" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C38" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D38" s="11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B39" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C39" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D39" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B40" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C40" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D40" s="11">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="41" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B41" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C41" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D41" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="42" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B42" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C42" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D42" s="11">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B43" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C43" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D43" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B44" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C44" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D44" s="11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="45" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B45" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C45" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D45" s="1">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="46" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B46" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C46" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D46" s="11">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="47" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B47" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C47" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D47" s="1">
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="48" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B48" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C48" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D48" s="11">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="49" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B49" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C49" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D49" s="1">
+        <v>22.5</v>
+      </c>
+    </row>
+    <row r="50" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B50" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C50" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D50" s="11">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="51" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B51" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C51" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D51" s="1">
+        <v>27.5</v>
+      </c>
+    </row>
+    <row r="52" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B52" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C52" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D52" s="11">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="53" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B53" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C53" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D53" s="1">
+        <v>32.5</v>
+      </c>
+    </row>
+    <row r="54" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B54" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C54" s="19" t="s">
+        <v>118</v>
+      </c>
+      <c r="D54" s="11">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="55" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B55" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C55" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="D55" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="56" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B56" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C56" s="19" t="s">
+        <v>118</v>
+      </c>
+      <c r="D56" s="11">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="57" spans="2:4" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B57" s="30" t="s">
+        <v>18</v>
+      </c>
+      <c r="C57" s="44" t="s">
+        <v>121</v>
+      </c>
+      <c r="D57" s="2">
+        <v>70</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B25:D25"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EED9BCF-AC84-402D-B7FA-16D351A40D85}">
   <dimension ref="B1:C7"/>
   <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -10477,10 +11045,10 @@
   <sheetData>
     <row r="1" spans="2:3" ht="16" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="2:3" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="141" t="s">
+      <c r="B2" s="144" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="142"/>
+      <c r="C2" s="145"/>
     </row>
     <row r="3" spans="2:3" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B3" s="5" t="s">
@@ -10528,382 +11096,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87885471-7CC2-479B-9C76-A0AAB2D0375D}">
-  <dimension ref="B1:H28"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="2" max="2" width="23.25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.75" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="40.25" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.25" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.83203125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B2" s="125" t="s">
-        <v>131</v>
-      </c>
-      <c r="C2" s="126"/>
-      <c r="D2" s="126"/>
-      <c r="E2" s="127"/>
-      <c r="G2" s="115" t="s">
-        <v>22</v>
-      </c>
-      <c r="H2" s="116">
-        <v>47.287930000000003</v>
-      </c>
-    </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B3" s="21" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="18" t="s">
-        <v>122</v>
-      </c>
-      <c r="D3" s="18" t="s">
-        <v>4</v>
-      </c>
-      <c r="E3" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="G3" s="101" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="117">
-        <v>-71.167720000000003</v>
-      </c>
-    </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B4" s="112" t="s">
-        <v>198</v>
-      </c>
-      <c r="C4" s="20" t="s">
-        <v>200</v>
-      </c>
-      <c r="D4" s="119" t="s">
-        <v>175</v>
-      </c>
-      <c r="E4" s="114" t="s">
-        <v>172</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="H4" s="113" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="5" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="32" t="s">
-        <v>199</v>
-      </c>
-      <c r="C5" s="20" t="s">
-        <v>201</v>
-      </c>
-      <c r="D5" s="120" t="s">
-        <v>175</v>
-      </c>
-      <c r="E5" s="114" t="s">
-        <v>172</v>
-      </c>
-      <c r="G5" s="103" t="s">
-        <v>162</v>
-      </c>
-      <c r="H5" s="111" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B6" s="32" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="20" t="s">
-        <v>108</v>
-      </c>
-      <c r="D6" s="120" t="s">
-        <v>171</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B7" s="32" t="s">
-        <v>209</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>206</v>
-      </c>
-      <c r="D7" s="120">
-        <v>1</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B8" s="32" t="s">
-        <v>207</v>
-      </c>
-      <c r="C8" s="20" t="s">
-        <v>206</v>
-      </c>
-      <c r="D8" s="120">
-        <v>2</v>
-      </c>
-      <c r="E8" s="1"/>
-    </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B9" s="32" t="s">
-        <v>208</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>206</v>
-      </c>
-      <c r="D9" s="120">
-        <v>1</v>
-      </c>
-      <c r="E9" s="14"/>
-    </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B10" s="32" t="s">
-        <v>180</v>
-      </c>
-      <c r="C10" s="20" t="s">
-        <v>126</v>
-      </c>
-      <c r="D10" s="121" t="s">
-        <v>182</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B11" s="32" t="s">
-        <v>181</v>
-      </c>
-      <c r="C11" s="20" t="s">
-        <v>126</v>
-      </c>
-      <c r="D11" s="121" t="s">
-        <v>184</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B12" s="32" t="s">
-        <v>197</v>
-      </c>
-      <c r="C12" s="20" t="s">
-        <v>113</v>
-      </c>
-      <c r="D12" s="120" t="s">
-        <v>202</v>
-      </c>
-      <c r="E12" s="118" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B13" s="32" t="s">
-        <v>196</v>
-      </c>
-      <c r="C13" s="20" t="s">
-        <v>113</v>
-      </c>
-      <c r="D13" s="120" t="s">
-        <v>203</v>
-      </c>
-      <c r="E13" s="114" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B14" s="32" t="s">
-        <v>194</v>
-      </c>
-      <c r="C14" s="20" t="s">
-        <v>113</v>
-      </c>
-      <c r="D14" s="120" t="s">
-        <v>204</v>
-      </c>
-      <c r="E14" s="114" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B15" s="32" t="s">
-        <v>195</v>
-      </c>
-      <c r="C15" s="20" t="s">
-        <v>113</v>
-      </c>
-      <c r="D15" s="120" t="s">
-        <v>205</v>
-      </c>
-      <c r="E15" s="114" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B16" s="32" t="s">
-        <v>185</v>
-      </c>
-      <c r="C16" s="20" t="s">
-        <v>128</v>
-      </c>
-      <c r="D16" s="120">
-        <v>-0.08</v>
-      </c>
-      <c r="E16" s="1"/>
-    </row>
-    <row r="17" spans="2:5" ht="31" x14ac:dyDescent="0.35">
-      <c r="B17" s="32" t="s">
-        <v>173</v>
-      </c>
-      <c r="C17" s="64" t="s">
-        <v>109</v>
-      </c>
-      <c r="D17" s="120" t="s">
-        <v>175</v>
-      </c>
-      <c r="E17" s="114" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="18" spans="2:5" ht="31" x14ac:dyDescent="0.35">
-      <c r="B18" s="32" t="s">
-        <v>174</v>
-      </c>
-      <c r="C18" s="64" t="s">
-        <v>125</v>
-      </c>
-      <c r="D18" s="120" t="s">
-        <v>175</v>
-      </c>
-      <c r="E18" s="114" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B19" s="32" t="s">
-        <v>176</v>
-      </c>
-      <c r="C19" s="20" t="s">
-        <v>114</v>
-      </c>
-      <c r="D19" s="120" t="s">
-        <v>175</v>
-      </c>
-      <c r="E19" s="14" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B20" s="32" t="s">
-        <v>177</v>
-      </c>
-      <c r="C20" s="20" t="s">
-        <v>114</v>
-      </c>
-      <c r="D20" s="120" t="s">
-        <v>175</v>
-      </c>
-      <c r="E20" s="14" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B21" s="32" t="s">
-        <v>192</v>
-      </c>
-      <c r="C21" s="20" t="s">
-        <v>111</v>
-      </c>
-      <c r="D21" s="120">
-        <v>8.5</v>
-      </c>
-      <c r="E21" s="14"/>
-    </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B22" s="32" t="s">
-        <v>193</v>
-      </c>
-      <c r="C22" s="20" t="s">
-        <v>111</v>
-      </c>
-      <c r="D22" s="120">
-        <v>14.6</v>
-      </c>
-      <c r="E22" s="14"/>
-    </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B23" s="32" t="s">
-        <v>187</v>
-      </c>
-      <c r="C23" s="20" t="s">
-        <v>127</v>
-      </c>
-      <c r="D23" s="120">
-        <v>2.5</v>
-      </c>
-      <c r="E23" s="14" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="24" spans="2:5" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B24" s="57" t="s">
-        <v>191</v>
-      </c>
-      <c r="C24" s="44" t="s">
-        <v>130</v>
-      </c>
-      <c r="D24" s="122">
-        <v>-0.04</v>
-      </c>
-      <c r="E24" s="59"/>
-    </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B26" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B27" s="144" t="s">
-        <v>190</v>
-      </c>
-      <c r="C27" s="144"/>
-      <c r="D27" s="144"/>
-      <c r="E27" s="144"/>
-    </row>
-    <row r="28" spans="2:5" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="143" t="s">
-        <v>189</v>
-      </c>
-      <c r="C28" s="143"/>
-      <c r="D28" s="143"/>
-      <c r="E28" s="143"/>
-    </row>
-  </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B4:E24">
-    <sortCondition ref="B4:B24"/>
-  </sortState>
-  <mergeCells count="3">
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B28:E28"/>
-    <mergeCell ref="B27:E27"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>